<commit_message>
CRWV 2026-10-14 evening: near-term financing map (Debt sheet block + page block) after the credit sell-off
- Template DCF CRWV.xlsx / build_crwv_model.py: 'Near-term financing map' on the Debt sheet — post-quarter DDTL 5.5 $2.6bn, $1.2bn revolver draw, 2.875% 2033 convert ($3.7bn priced / $4.2bn per DB; GS indicative terms 09-17), 35m-share ATM; NTM sources 22.4bn vs uses 41.6bn -> ~$19bn residual; DB/UBS cross-checks; 10-14 bond/CDS/equity levels. DCF unchanged ($59.01).
- CRWV.md: dated block at the head of Current state (tape, DB Zelnick Buy $150 note, the house map) + Changelog. No Barclays CRWV e-mail found today (connector + Outlook COM scan); last Barclays note on file remains Lenschow/McMeans 2026-09-17.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_wiki/_data/research/CRWV_official_model_2026-10-14/Template DCF CRWV.xlsx
+++ b/_wiki/_data/research/CRWV_official_model_2026-10-14/Template DCF CRWV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Wiki Felipe empresas\_wiki\_data\research\CRWV_official_model_2026-10-14\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03BDB17-08A6-4A65-BB40-3FA6AFC32B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328DF53D-2614-43D2-9550-1574C8F12F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="481">
   <si>
     <t>CRWV | Power-driven DCF (IT-load GW x revenue per GW)</t>
   </si>
@@ -1290,6 +1290,195 @@
   </si>
   <si>
     <t>Subsequent events (10-Q 2Q26 note 16): Aug-26 $2.6bn DDTL 5.5 (JPMorgan agent; SOFR+550, matures Sep-31) and a $1.2bn draw on the Revolving Credit Facility — NOT in the model's 30-Jun-26 net debt (the draw funds 2H26 capex already discounted in the FCFF).</t>
+  </si>
+  <si>
+    <t>Near-term financing map | 3Q26 → 2Q27 (NTM) — mapped 2026-10-14 (CRWV bonds at 14.5-15.7%, equity −15.5% on the day)</t>
+  </si>
+  <si>
+    <t>Post-quarter financing (after the 30-Jun-26 balance sheet) — NOT in the model's net debt (valuation date 30-Jun-26; the convert is cash-neutral net of capped calls)</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Aug-2026</t>
+  </si>
+  <si>
+    <t>DDTL 5.5 ($2.6bn facility; SOFR + 5.50%; matures Sep-2031; backed by shorter 3-yr contracts)</t>
+  </si>
+  <si>
+    <t>10-Q 2Q26 note 16 (subsequent events); DB Zelnick 2026-10-14; Redburn 09-21 Fig 70.</t>
+  </si>
+  <si>
+    <t>Revolving Credit Facility draw (within the $10.0bn undrawn availability at 30-Jun — not new capacity)</t>
+  </si>
+  <si>
+    <t>10-Q 2Q26 note 16.</t>
+  </si>
+  <si>
+    <t>Sep-2026</t>
+  </si>
+  <si>
+    <t>2.875% Convertible Senior Notes due Apr-2033: $3.0bn + $0.5bn greenshoe indicative (coupon 2.375-2.875%, premium 22.5-27.5%, capped calls), priced $3.7bn on 09-18; DB counts $4.2bn</t>
+  </si>
+  <si>
+    <t>GS bookrunner indicative terms 2026-09-17; The Information 2026-09-20 ($3.7bn priced, above target); DB Zelnick 2026-10-14 ($4.2bn 2.875%). Final conversion price not captured — out of the money at $65.78.</t>
+  </si>
+  <si>
+    <t>ATM equity programme, 35m shares — registered, NOT used ('not at these prices', Robbins 09-21); ~$2.3bn at $65.78</t>
+  </si>
+  <si>
+    <t>Barclays Lenschow 2026-09-17 (structure); BTG websession 2026-09-21 (lock-up + blackout until after the 3Q26 call).</t>
+  </si>
+  <si>
+    <t>New debt capital raised after 30-Jun (DDTL 5.5 + convert; revolver draw excluded as it sat inside the undrawn availability)</t>
+  </si>
+  <si>
+    <t>Sources vs uses, next twelve months (US$ m) — model basis unless noted; FCFF is pre-interest</t>
+  </si>
+  <si>
+    <t>Line</t>
+  </si>
+  <si>
+    <t>Basis / source</t>
+  </si>
+  <si>
+    <t>Total liquidity at 30-Jun-26 (cash 5,524 + securities 15 + undrawn facilities 10,014)</t>
+  </si>
+  <si>
+    <t>10-Q 2Q26 'Liquidity and Capital Resources' table: $15,553m.</t>
+  </si>
+  <si>
+    <t>New debt capital after 30-Jun (DDTL 5.5 + 2033 convert)</t>
+  </si>
+  <si>
+    <t>Table above.</t>
+  </si>
+  <si>
+    <t>Sources available (liquidity + new capital)</t>
+  </si>
+  <si>
+    <t>1H26 free cash flow, company basis (EBITDA 2,710 − SBC 318 − capex 16,200 + NWC inflow ~2,135)</t>
+  </si>
+  <si>
+    <t>10-Q 2Q26 cash flow + calls (capex company basis); double-check reconstruction 2026-10-14.</t>
+  </si>
+  <si>
+    <t>2H26 FCFF = FY26 model FCFF − 1H26 actual</t>
+  </si>
+  <si>
+    <t>Model: FY26 FCFF (cover) less 1H26 actual.</t>
+  </si>
+  <si>
+    <t>1H27 FCFF = half of the model's 2027 FCFF</t>
+  </si>
+  <si>
+    <t>Model 2027 FCFF (cover) ÷ 2.</t>
+  </si>
+  <si>
+    <t>Cash interest NTM: 2H26 (3Q guide $860-940m + 4Q ~1,000) + 1H27 (half of model 2027)</t>
+  </si>
+  <si>
+    <t>Call 2026-08-11 (3Q guide); model 2027 net interest (cover memo block).</t>
+  </si>
+  <si>
+    <t>Scheduled principal NTM: remainder of 2026 (4,413) + half of 2027 (6,184)</t>
+  </si>
+  <si>
+    <t>10-Q 2Q26 note 10 principal schedule.</t>
+  </si>
+  <si>
+    <t>Uses NTM (FCFF 2H26 + 1H27 + interest + principal)</t>
+  </si>
+  <si>
+    <t>Residual to raise over the NTM (sources + uses; negative = still to fund)</t>
+  </si>
+  <si>
+    <t>Funded in practice by project DDTLs drawn against backlog as capex lands (UBS: DDTLs fund ~90% of capex) — the gap is a flow, not a liquidity hole on day one.</t>
+  </si>
+  <si>
+    <t>Cross-checks from other houses (same window, different bases)</t>
+  </si>
+  <si>
+    <t>DB Zelnick 2026-10-14: NTM OCF ~$10bn vs required capex ~$45bn → ~$35bn pre-debt-service gap; 'available liquidity $15.5bn exiting C2Q'; Buy PT $150</t>
+  </si>
+  <si>
+    <t>DB 2-page note (e-mail body archived to _inbox 2026-10-14). OCF basis = after interest; capex company basis.</t>
+  </si>
+  <si>
+    <t>UBS Keirstead 2026-09-22: cumulative 2027-30 capex ~$260bn vs OCF ~$158bn → ~$102bn of additional financing 2027-30</t>
+  </si>
+  <si>
+    <t>UBS initiation p.-; 4-year window, not NTM.</t>
+  </si>
+  <si>
+    <t>Model: cumulative FCFF 2027-30 (pre-interest) + interest 2027-30</t>
+  </si>
+  <si>
+    <t>Cover rows; compare with UBS's $102bn (model is more punitive: smaller prepayment inflows, 9% on the whole balance).</t>
+  </si>
+  <si>
+    <t>FT 2026-10-14 (co-founder McBee): courting insurers' 'unlimited' capital via investment-grade, chip-backed loans — the next funding pool after DDTLs</t>
+  </si>
+  <si>
+    <t>FT via Jefferies (Wong) / UBS desk (Ruple) / Vital Knowledge, 2026-10-14; TMTB EOD wrap. Reported, not a filed facility.</t>
+  </si>
+  <si>
+    <t>CEO staff memo 2026-10-14 (Bloomberg, via TMTB): backlog 'more than supports' the debt; market acting 'irrationally'</t>
+  </si>
+  <si>
+    <t>Management characterisation relayed by a newsletter — not a filing.</t>
+  </si>
+  <si>
+    <t>Market levels 2026-10-14 (credit monitor, Bloomberg YLD_YTM_MID / PX_LAST; desks for the CDS print)</t>
+  </si>
+  <si>
+    <t>CoreWeave 9.25% Jun-2030 yield</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>CoreWeave 9.00% Feb-2031 yield</t>
+  </si>
+  <si>
+    <t>CoreWeave 9.75% Oct-2031 yield</t>
+  </si>
+  <si>
+    <t>CoreWeave 9.625% Jul-2032 yield</t>
+  </si>
+  <si>
+    <t>CoreWeave 8.5% Jul-2032 EUR yield</t>
+  </si>
+  <si>
+    <t>Convertible 1.75% Dec-2031 yield</t>
+  </si>
+  <si>
+    <t>Convertible 1.75% Oct-2032 yield</t>
+  </si>
+  <si>
+    <t>Convertible 2.875% Apr-2033 yield</t>
+  </si>
+  <si>
+    <t>5Y CDS — Bloomberg D14 quote (bp)</t>
+  </si>
+  <si>
+    <t>bp</t>
+  </si>
+  <si>
+    <t>5Y CDS — desks (Rothschild TMT daily 10-14, @zerohedge; 'almost 1,000bp', TMTB) (bp)</t>
+  </si>
+  <si>
+    <t>Equity close 2026-10-14 (BBG; −15.5% on the day per TMTB)</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Basis warning: the Bloomberg D14 CDS quote (440bp) and the desk prints (~1,000bp, 'pricing a ~58% 5-year default probability' per TMTB) are different quotes/contracts — not reconciled here; the bonds at 14.5-15.7% are the cleaner observable. The 2032 unsecureds traded below 80c (TMTB).</t>
+  </si>
+  <si>
+    <t>No Barclays research on CoreWeave reached the mailbox on 2026-10-14 (only the TMT desk flow list names CRWV). Barclays' last CRWV note on file: Lenschow/McMeans 2026-09-17, EW PT $105 (the convert + ATM structure).</t>
   </si>
 </sst>
 </file>
@@ -10475,7 +10664,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="C2:H44"/>
+  <dimension ref="C2:H88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="2.28515625" customWidth="1"/>
@@ -10951,7 +11140,7 @@
         <v>6184</v>
       </c>
     </row>
-    <row r="33" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D33" s="5" t="s">
         <v>407</v>
       </c>
@@ -10959,7 +11148,7 @@
         <v>4416</v>
       </c>
     </row>
-    <row r="34" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D34" s="5" t="s">
         <v>408</v>
       </c>
@@ -10967,7 +11156,7 @@
         <v>2421</v>
       </c>
     </row>
-    <row r="35" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D35" s="5" t="s">
         <v>409</v>
       </c>
@@ -10975,7 +11164,7 @@
         <v>3221</v>
       </c>
     </row>
-    <row r="36" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D36" s="5" t="s">
         <v>410</v>
       </c>
@@ -10983,7 +11172,7 @@
         <v>14896</v>
       </c>
     </row>
-    <row r="37" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D37" s="20" t="s">
         <v>411</v>
       </c>
@@ -10992,34 +11181,454 @@
         <v>35551</v>
       </c>
     </row>
-    <row r="39" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D39" s="69" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="40" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D40" s="69" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="41" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D41" s="69" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="42" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D42" s="69" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="43" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D43" s="69" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="44" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D44" s="69" t="s">
         <v>417</v>
+      </c>
+    </row>
+    <row r="46" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D46" s="10" t="s">
+        <v>418</v>
+      </c>
+      <c r="E46" s="11"/>
+      <c r="F46" s="11"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
+    </row>
+    <row r="47" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D47" s="20" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="48" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C48" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="49" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C49" s="71" t="s">
+        <v>421</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E49" s="50">
+        <v>2600</v>
+      </c>
+      <c r="F49" s="69" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="50" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C50" s="71" t="s">
+        <v>421</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="E50" s="50">
+        <v>1200</v>
+      </c>
+      <c r="F50" s="69" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="51" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C51" s="71" t="s">
+        <v>426</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="E51" s="50">
+        <v>4200</v>
+      </c>
+      <c r="F51" s="69" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="52" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C52" s="71" t="s">
+        <v>426</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="E52" s="50">
+        <v>0</v>
+      </c>
+      <c r="F52" s="69" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="53" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D53" s="20" t="s">
+        <v>431</v>
+      </c>
+      <c r="E53" s="21">
+        <f>E49+E51</f>
+        <v>6800</v>
+      </c>
+    </row>
+    <row r="55" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D55" s="20" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="56" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C56" s="4"/>
+      <c r="D56" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="57" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D57" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="E57" s="50">
+        <v>15553</v>
+      </c>
+      <c r="F57" s="69" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="58" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D58" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="E58" s="13">
+        <f>E53</f>
+        <v>6800</v>
+      </c>
+      <c r="F58" s="69" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="59" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D59" s="20" t="s">
+        <v>439</v>
+      </c>
+      <c r="E59" s="21">
+        <f>E57+E58</f>
+        <v>22353</v>
+      </c>
+      <c r="F59" s="69"/>
+    </row>
+    <row r="60" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D60" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="E60" s="50">
+        <v>-11673</v>
+      </c>
+      <c r="F60" s="69" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="61" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D61" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="E61" s="13">
+        <f>'DCF Cover - Base'!G46-E60</f>
+        <v>-14682.75</v>
+      </c>
+      <c r="F61" s="69" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="62" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D62" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="E62" s="13">
+        <f>'DCF Cover - Base'!H46/2</f>
+        <v>-14808.825000000001</v>
+      </c>
+      <c r="F62" s="69" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="63" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D63" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="E63" s="13">
+        <f>-(1900+'DCF Cover - Base'!H105/2)</f>
+        <v>-4607.6874906249996</v>
+      </c>
+      <c r="F63" s="69" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="64" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D64" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="E64" s="50">
+        <v>-7505</v>
+      </c>
+      <c r="F64" s="69" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="65" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D65" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="E65" s="21">
+        <f>SUM(E61:E64)</f>
+        <v>-41604.262490624998</v>
+      </c>
+      <c r="F65" s="69"/>
+    </row>
+    <row r="66" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D66" s="20" t="s">
+        <v>451</v>
+      </c>
+      <c r="E66" s="21">
+        <f>E59+E65</f>
+        <v>-19251.262490624998</v>
+      </c>
+      <c r="F66" s="69" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="68" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D68" s="20" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="69" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D69" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="E69" s="50">
+        <v>-35000</v>
+      </c>
+      <c r="F69" s="69" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="70" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D70" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="E70" s="50">
+        <v>-102000</v>
+      </c>
+      <c r="F70" s="69" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="71" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D71" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="E71" s="13">
+        <f>SUM('DCF Cover - Base'!H46:K46)-SUM('DCF Cover - Base'!H105:K105)</f>
+        <v>-139351.00954221789</v>
+      </c>
+      <c r="F71" s="69" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="72" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D72" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="E72" s="50">
+        <v>0</v>
+      </c>
+      <c r="F72" s="69" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="73" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D73" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="E73" s="50">
+        <v>0</v>
+      </c>
+      <c r="F73" s="69" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="75" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D75" s="20" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="76" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D76" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="E76" s="51">
+        <v>14.46</v>
+      </c>
+      <c r="F76" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="77" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D77" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="E77" s="51">
+        <v>15</v>
+      </c>
+      <c r="F77" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="78" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D78" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="E78" s="51">
+        <v>15.69</v>
+      </c>
+      <c r="F78" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="79" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D79" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="E79" s="51">
+        <v>15.56</v>
+      </c>
+      <c r="F79" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="80" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D80" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="E80" s="51">
+        <v>14.46</v>
+      </c>
+      <c r="F80" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="81" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D81" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="E81" s="51">
+        <v>6.56</v>
+      </c>
+      <c r="F81" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="82" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D82" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E82" s="51">
+        <v>7.78</v>
+      </c>
+      <c r="F82" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="83" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D83" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="E83" s="51">
+        <v>5.75</v>
+      </c>
+      <c r="F83" s="69" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="84" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D84" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="E84" s="50">
+        <v>440</v>
+      </c>
+      <c r="F84" s="69" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="85" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D85" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="E85" s="50">
+        <v>1000</v>
+      </c>
+      <c r="F85" s="69" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="86" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D86" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="E86" s="51">
+        <v>65.78</v>
+      </c>
+      <c r="F86" s="69" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="87" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D87" s="69" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="88" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D88" s="69" t="s">
+        <v>480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>